<commit_message>
Incluir 142030 com o hospede confirmado e fechar os lotes submetidos
O utilizador confirmou que o hospede da fatura 142030 e HEEKYUNG CHOI. As
observacoes do InvoiceXpress traziam ali o nome da propria agencia, o que
levou a reter a fatura na versao anterior deste lote. Com o nome confirmado a
fatura entra no lote, que passa de 27 para 28 faturas, de 41 para 43 linhas e
de 4.720,19 para 4.974,04 EUR. Passa a cobrir a totalidade das faturas
Hotelbeds emitidas no intervalo. A 142030 leva um acerto de um centimo na
ultima linha, como as outras seis.

A versao retida nunca chegou a ser carregada, pelo que a substituicao nao
duplica nada no portal.

Os lotes 07-08/13-08 e 14-08/17-08 foram confirmados como carregados e as
suas 18 faturas passam de 'prepared' a 'uploaded'. Fica apenas este lote por
submeter.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011KuDsfLuFb1wQzTRo3ZDUs
</commit_message>
<xml_diff>
--- a/hotelbeds_18-08_31-08_revisao.xlsx
+++ b/hotelbeds_18-08_31-08_revisao.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,12 +33,8 @@
     <font>
       <b val="1"/>
     </font>
-    <font>
-      <b val="1"/>
-      <color rgb="009C5700"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -48,11 +44,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="004472C4"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -68,13 +59,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -441,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J31"/>
+  <dimension ref="A1:J30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1751,70 +1741,70 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr"/>
-      <c r="B29" s="2" t="inlineStr"/>
-      <c r="C29" s="2" t="inlineStr"/>
-      <c r="D29" s="2" t="inlineStr"/>
-      <c r="E29" s="2" t="inlineStr"/>
-      <c r="F29" s="2" t="inlineStr">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>142030</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>267387537</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>18-08-2026</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>18-08-2026</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>HEEKYUNG CHOI</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>59-5970070</t>
+        </is>
+      </c>
+      <c r="G29" t="n">
+        <v>2</v>
+      </c>
+      <c r="H29" t="n">
+        <v>253.85</v>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>0,01</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>prepared</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr"/>
+      <c r="B30" s="2" t="inlineStr"/>
+      <c r="C30" s="2" t="inlineStr"/>
+      <c r="D30" s="2" t="inlineStr"/>
+      <c r="E30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="G29" s="2" t="n">
-        <v>41</v>
-      </c>
-      <c r="H29" s="2" t="n">
-        <v>4720.190000000001</v>
-      </c>
-      <c r="I29" s="2" t="inlineStr"/>
-      <c r="J29" s="2" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="3" t="inlineStr">
-        <is>
-          <t>142030</t>
-        </is>
-      </c>
-      <c r="B31" s="3" t="n">
-        <v>267387537</v>
-      </c>
-      <c r="C31" s="3" t="inlineStr">
-        <is>
-          <t>18-08-2026</t>
-        </is>
-      </c>
-      <c r="D31" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E31" s="3" t="inlineStr">
-        <is>
-          <t>(sem nome de hóspede)</t>
-        </is>
-      </c>
-      <c r="F31" s="3" t="inlineStr">
-        <is>
-          <t>59-5970070</t>
-        </is>
-      </c>
-      <c r="G31" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="H31" s="3" t="n">
-        <v>253.85</v>
-      </c>
-      <c r="I31" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J31" s="3" t="inlineStr">
-        <is>
-          <t>RETIDA</t>
-        </is>
-      </c>
+      <c r="G30" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="H30" s="2" t="n">
+        <v>4974.040000000001</v>
+      </c>
+      <c r="I30" s="2" t="inlineStr"/>
+      <c r="J30" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1827,7 +1817,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J42"/>
+  <dimension ref="A1:J44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1843,52 +1833,52 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Nº Fatura</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Hóspede</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>Booking Nº</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Data do serviço (noite)</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Noites</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>Qtd</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>Preço c/IVA</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>Total linha</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>IVA %</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>Moeda</t>
         </is>
@@ -3611,6 +3601,90 @@
         <v>6</v>
       </c>
       <c r="J42" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>142030</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>HEEKYUNG CHOI</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>59-5970070</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>16-08-2026</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>1</v>
+      </c>
+      <c r="F43" t="n">
+        <v>1</v>
+      </c>
+      <c r="G43" t="n">
+        <v>126.92</v>
+      </c>
+      <c r="H43" t="n">
+        <v>126.92</v>
+      </c>
+      <c r="I43" t="n">
+        <v>6</v>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>142030</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>HEEKYUNG CHOI</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>59-5970070</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>17-08-2026</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>1</v>
+      </c>
+      <c r="F44" t="n">
+        <v>1</v>
+      </c>
+      <c r="G44" t="n">
+        <v>126.93</v>
+      </c>
+      <c r="H44" t="n">
+        <v>126.93</v>
+      </c>
+      <c r="I44" t="n">
+        <v>6</v>
+      </c>
+      <c r="J44" t="inlineStr">
         <is>
           <t>EUR</t>
         </is>

</xml_diff>